<commit_message>
data: 2026-06-26 일별 수집
</commit_message>
<xml_diff>
--- a/data/daily/2026-06-26.xlsx
+++ b/data/daily/2026-06-26.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="카카오선물하기" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="다이소몰" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="올리브영" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="카카오선물하기" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="다이소몰" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="카테고리통계" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,13 +19,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -36,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -44,12 +47,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,41 +430,41 @@
   <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="59" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="43" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>순위</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>상품명</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>브랜드</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>가격</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>상품URL</t>
         </is>
@@ -461,7 +473,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>건강식품·영양제</t>
+          <t>멀티비타민/종합비타민</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -469,29 +481,29 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>[카카오 단독 특가]센트룸 원데이팩 맨/우먼 2030 30일팩 2종 택1</t>
+          <t>오쏘몰 이뮨 멀티비타민&amp;미네랄 7입 (공식수입)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>센트룸</t>
+          <t>오쏘몰</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>50,000원</t>
+          <t>34,000원</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/10591119</t>
+          <t>https://gift.kakao.com/product/2301047</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>건강식품·영양제</t>
+          <t>멀티비타민/종합비타민</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -499,29 +511,29 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>오쏘몰 이뮨 멀티비타민&amp;미네랄 7입 (공식수입)</t>
+          <t>옵티젠 이뮨 멀티비타민&amp;미네랄 10입 / 1박스 (+GIFT 쇼핑백)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>단독</t>
+          <t>옵티젠</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>34,000원</t>
+          <t>26,900원</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/2301047</t>
+          <t>https://gift.kakao.com/product/7608679</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>건강식품·영양제</t>
+          <t>멀티비타민/종합비타민</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -529,29 +541,29 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>옵티젠 이뮨 멀티비타민&amp;미네랄 10입 / 1박스 (+GIFT 쇼핑백)</t>
+          <t>오쏘몰 이뮨 멀티비타민&amp;미네랄 10입(7+3) - 스페셜 기프트 에디션 (공식수입)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>옵티젠</t>
+          <t>오쏘몰</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>26,900원</t>
+          <t>43,000원</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/7608679</t>
+          <t>https://gift.kakao.com/product/11866425</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>건강식품·영양제</t>
+          <t>멀티비타민/종합비타민</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -559,7 +571,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>오쏘몰 이뮨 멀티비타민&amp;미네랄 10입(7+3) - 스페셜 기프트 에디션 (공식수입)</t>
+          <t>오쏘몰 이뮨 멀티비타민&amp;미네랄 30입 - 시그니처 기프트 에디션 (공식수입)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -569,19 +581,19 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>43,000원</t>
+          <t>109,000원</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/11866425</t>
+          <t>https://gift.kakao.com/product/2484405</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>건강식품·영양제</t>
+          <t>멀티비타민/종합비타민</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -589,29 +601,29 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>오쏘몰 이뮨 멀티비타민&amp;미네랄 30입 - 시그니처 기프트 에디션 (공식수입)</t>
+          <t>[센트룸] 맛있는 멀티비타민 미네랄 멀티구미 (80구미)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>오쏘몰</t>
+          <t>센트룸</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>109,000원</t>
+          <t>24,000원</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/2484405</t>
+          <t>https://gift.kakao.com/product/7320451</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>건강식품·영양제</t>
+          <t>멀티비타민/종합비타민</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -619,29 +631,29 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>[센트룸] 맛있는 멀티비타민 미네랄 멀티구미 (80구미)</t>
+          <t>뉴트리포유 듀얼+ 이뮨 종합 멀티비타민&amp;미네랄 7입+2입 증정 - 선물하기 단독 에디션</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>단독</t>
+          <t>뉴트리포유</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>24,000원</t>
+          <t>19,900원</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/7320451</t>
+          <t>https://gift.kakao.com/product/10056171</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>건강식품·영양제</t>
+          <t>홍삼/인삼</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -649,29 +661,29 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>뉴트리포유 듀얼+ 이뮨 종합 멀티비타민&amp;미네랄 7입+2입 증정 - 선물하기 단독 에디션</t>
+          <t>[정관장] 활기마이트(액상30ml+분말500mg) 7병 + [증정] 여행용 화장품 키트</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>뉴트리포유</t>
+          <t>정관장</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>19,900원</t>
+          <t>35,000원</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/10056171</t>
+          <t>https://gift.kakao.com/product/12159594</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>건강식품·영양제</t>
+          <t>멀티비타민/종합비타민</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -679,29 +691,29 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>[정관장] 활기마이트(액상30ml+분말500mg) 7병 + [증정] 여행용 화장품 키트</t>
+          <t>이뮨 멀티비타민 미네랄 7입+비타민젤리 마시는 액상 종합 비타민 수험생 직장인 부모님 건강 선물</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>단독</t>
+          <t>종근당</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>35,000원</t>
+          <t>23,800원</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/12159594</t>
+          <t>https://gift.kakao.com/product/7948462</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>건강식품·영양제</t>
+          <t>멀티비타민/종합비타민</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -709,29 +721,29 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>이뮨 멀티비타민 미네랄 7입+비타민젤리 마시는 액상 종합 비타민 수험생 직장인 부모님 건강 선물</t>
+          <t>아임비타 멀티비타민 이뮨샷 1박스(5입) / 비타민선물 응원선물 에너지 선물 직장동료 선물</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>종근당</t>
+          <t>종근당건강</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>23,800원</t>
+          <t>15,900원</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/7948462</t>
+          <t>https://gift.kakao.com/product/5551542</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>건강식품·영양제</t>
+          <t>비타민C/항산화</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -739,29 +751,29 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>아임비타 멀티비타민 이뮨샷 1박스(5입) / 비타민선물 응원선물 에너지 선물 직장동료 선물</t>
+          <t>고려은단 메가도스C 3000 100포 / 분말비타민C</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>종근당건강</t>
+          <t>고려은단</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>15,900원</t>
+          <t>24,900원</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/5551542</t>
+          <t>https://gift.kakao.com/product/3252731</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>다이어트·이너뷰티</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -769,29 +781,29 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>물에 타먹는 발포형 무설탕 이온음료 요헤미티 워터 네가지 맛 4통(40정)</t>
+          <t>[그레인온] 골드 카무트 브랜드밀 효소 3개월(+선물포장)+파인키위효소 1개월+저당견과류바</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>요헤미티</t>
+          <t>그레인온</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>34,000원</t>
+          <t>43,900원</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/13372860</t>
+          <t>https://gift.kakao.com/product/13180343</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>다이어트·이너뷰티</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -799,29 +811,29 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>[그레인온] 골드 카무트 브랜드밀 효소 3개월(+선물포장)+파인키위효소 1개월+저당견과류바</t>
+          <t>[한끼통살] 닭가슴살 한달 식단패키지 30팩+(증정)보냉백</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>그레인온</t>
+          <t>한끼통살</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>43,900원</t>
+          <t>45,900원</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/13180343</t>
+          <t>https://gift.kakao.com/product/11566779</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>다이어트·이너뷰티</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -851,7 +863,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>다이어트·이너뷰티</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -859,29 +871,29 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>[한끼통살] 닭가슴살 한달 식단패키지 30팩+(증정)보냉백</t>
+          <t>[한끼통살] 단백질 든든형 닭가슴살 21일 식단관리+(증정)전자레인지 용기</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>단독</t>
+          <t>한끼통살</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>45,900원</t>
+          <t>34,900원</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/11566779</t>
+          <t>https://gift.kakao.com/product/12860133</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>다이어트·이너뷰티</t>
+          <t>피부/미용</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -889,29 +901,29 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>[한끼통살] 단백질 든든형 닭가슴살 21일 식단관리+(증정)전자레인지 용기</t>
+          <t>"선물하기 1등 콜라겐" 아일로 타입1 콜라겐 비오틴 앰플 28일분 오간자 에디션+ 1입 추가 증정</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>한끼통살</t>
+          <t>아일로</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>34,900원</t>
+          <t>65,900원</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/12860133</t>
+          <t>https://gift.kakao.com/product/4965835</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>다이어트·이너뷰티</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -919,29 +931,29 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>"선물하기 1등 콜라겐" 아일로 타입1 콜라겐 비오틴 앰플 28일분 오간자 에디션+ 1입 추가 증정</t>
+          <t>[김종국 추천세트]익스트림 아르기닌정 (2개월분) &amp; 밀크씨슬 플러스 (2개월분) + 쇼핑백 증정</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>아일로</t>
+          <t>익스트림</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>65,900원</t>
+          <t>24,900원</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/4965835</t>
+          <t>https://gift.kakao.com/product/7556791</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>다이어트·이너뷰티</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -971,7 +983,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>다이어트·이너뷰티</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1001,7 +1013,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>다이어트·이너뷰티</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1009,29 +1021,29 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>식물성 멜라토닌 1mg 구미 젤리 멜라메이트 1박스 (20구미) 수험생/직장인 선물</t>
+          <t>셀렉스 프로핏 맛있는 완전단백질 250ml 18팩 딸기초코/모카초콜릿/밀크바닐라/바나나+베리오트바 2입 증정</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>CJ웰케어</t>
+          <t>셀렉스</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>8,900원</t>
+          <t>27,900원</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/11190137</t>
+          <t>https://gift.kakao.com/product/13550266</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>다이어트·이너뷰티</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1039,22 +1051,22 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>[운동선물/헬스] 삼대오백 모노 크레아틴 100서빙 운동 필수템</t>
+          <t>식물성 멜라토닌 1mg 구미 젤리 멜라메이트 1박스 (20구미) 수험생/직장인 선물</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>삼대오백</t>
+          <t>CJ웰케어</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>17,900원</t>
+          <t>8,900원</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/6352718</t>
+          <t>https://gift.kakao.com/product/11190137</t>
         </is>
       </c>
     </row>
@@ -1072,41 +1084,41 @@
   <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>순위</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>상품명</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>브랜드</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>가격</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>상품URL</t>
         </is>
@@ -1115,25 +1127,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>다이어트 홀릭 15일분</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>다이소</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+          <t>오브맘</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>5,000원</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=913624075&amp;recmYn=N</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -1141,21 +1165,29 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>신상 NEW</t>
+          <t>데일리와이즈 푸룬 구미 7일분</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>다이소</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
+          <t>종근당</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1,000원</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=032306208&amp;recmYn=N</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -1163,39 +1195,59 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>정성담은 배도라지스틱 12포</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>다이소</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
+          <t>자연관</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>5,000원</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=901762093&amp;recmYn=N</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>비타민D</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>4</v>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>비타민D＆아연 하루구미 30일분</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>다이소</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
+          <t>오브맘</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>5,000원</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=613602130&amp;recmYn=N</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -1203,21 +1255,29 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>음료/커피/차</t>
+          <t>콘드로이친 30정 30일분</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>다이소</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
+          <t>대웅제약</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>5,000원</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000152&amp;recmYn=N</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>비타민C/항산화</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -1225,21 +1285,29 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>사탕/초콜릿/젤리</t>
+          <t>리포좀 비타민C 30정</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>다이소</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
+          <t>동국제약</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>5,000원</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=610910679&amp;recmYn=N</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -1247,21 +1315,29 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>견과류/포</t>
+          <t>동국 맛있는 샐러드 미니볼 비타 15포 15일분</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>다이소</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
+          <t>동국제약</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>3,000원</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=610910967&amp;recmYn=N</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>마그네슘</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -1269,21 +1345,29 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>라면/즉석식품</t>
+          <t>마그네슘 30정 30일분</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>다이소</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
+          <t>대웅제약</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>3,000원</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000128&amp;recmYn=N</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>피부/미용</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -1291,34 +1375,54 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>기타식품</t>
+          <t>LG생활건강 이너뷰 콜라겐 더마스틱 7포</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>다이소</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
+          <t>이너뷰 바이 리튠</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>5,000원</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=994953528&amp;recmYn=N</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>10</v>
       </c>
-      <c r="C11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>락토핏 간케어 20포</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>다이소</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
+          <t>종근당건강</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>5,000원</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=591580891&amp;recmYn=N</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1331,347 +1435,311 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>순위</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>상품명</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>가격</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>상품URL</t>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>비율(%)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>카카오선물하기</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>다이소몰</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>올리브영</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>멀티비타민/종합비타민</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>[6월 올영픽] CJ 이너비 슬리밍 쾌변 젤리 벨리곰 기획 12포 (12일분)</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>CJ이너비</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>14,900원</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000254397</t>
-        </is>
+        <v>8</v>
+      </c>
+      <c r="C2" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="D2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>비타민C/항산화</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>2</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>빌드 프리미엄 테프 효소 /효소 유산균 30포 (1개월분)</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>빌드</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>15,900원</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000235606</t>
-        </is>
+      <c r="C3" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>비타민D</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>[10일콜라겐/모공,목주름/PDRN] 라이필 더마콜라겐 시그니처RN (10일분)</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>라이필</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>15,840원</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000259411</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="C4" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>마그네슘</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>[덴프스] 덴마크 유산균이야기 우먼 2개월분(질유산균) + 철분 헤모케어 3포 증정</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>덴프스</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>37,050원</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000202658</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="C5" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>루테인/눈건강</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>[단독선론칭] 에버콜라겐X민카롱 워터풀앰플 14포 2/6/12박스 (4/12/24주분)</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>에버콜라겐</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>29,700원</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=B000000260246</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>혈행</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>6</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>[1등 유산균] 콜레올로지 컷 다이어트 유산균 14/20캡슐 (7/10일분)</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>푸드올로지</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>18,500원</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000229934</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>홍삼/인삼</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>7</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>고려은단 비타민C1000 600정 (20개월분)</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>고려은단</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>42,900원</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000225938</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="C8" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>8</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>[서현PICK] 콜레올로지 PRO 600mg*30/60정 단품</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>푸드올로지</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>17,400원</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000175634</t>
-        </is>
+        <v>7</v>
+      </c>
+      <c r="C9" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="D9" t="n">
+        <v>6</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>프로바이오틱스/유산균</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>9</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>CJ 이너비 슬리밍 쾌변 젤리 벨리곰 기획 12포(+벨리곰 부적) / 단품</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>CJ이너비</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>14,900원</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000258608</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>건강식품</t>
+          <t>피부/미용</t>
         </is>
       </c>
       <c r="B11" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>기타/특수목적</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>8</v>
+      </c>
+      <c r="C12" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="D12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" t="n">
+        <v>5</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>합계</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>30</v>
+      </c>
+      <c r="C13" t="n">
+        <v>100</v>
+      </c>
+      <c r="D13" t="n">
+        <v>20</v>
+      </c>
+      <c r="E13" t="n">
         <v>10</v>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>[올영단독] 지노마스터 질유산균 70캡슐 (70일분)</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>지노마스터</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>59,000원</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000249509</t>
-        </is>
+      <c r="F13" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: 올리브영 impersonate chrome124→131 / 6/26~28 올리브영 데이터 백필
</commit_message>
<xml_diff>
--- a/data/daily/2026-06-26.xlsx
+++ b/data/daily/2026-06-26.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="카카오선물하기" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="다이소몰" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="카테고리통계" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="올리브영" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="카테고리통계" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,16 +20,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -39,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -47,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -439,32 +428,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>순위</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>상품명</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>브랜드</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>가격</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>상품URL</t>
         </is>
@@ -1093,32 +1082,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>순위</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>상품명</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>브랜드</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>가격</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>상품URL</t>
         </is>
@@ -1430,6 +1419,360 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>카테고리</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>순위</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>상품명</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>가격</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>상품URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>비타민C/항산화</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>고려은단 비타민C1000 이지+비타민D 120정 (60일분)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>고려은단</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>10,900원</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000164736&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>피부/미용</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>[10일콜라겐/모공,목주름/PDRN] 라이필 더마콜라겐 시그니처RN (10일분)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>라이필</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>15,840원</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000259411&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>기타/특수목적</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>레놉티 시너업글로우 14포 (14일분)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>레놉티</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>32,200원</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000222705&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=3</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>기타/특수목적</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>고려은단 메가도스 이뮨샷 4개입 (4일분)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>고려은단</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>9,900원</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000224748&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=4</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>프로바이오틱스/유산균</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>[덴프스] 덴마크 유산균이야기 우먼 2개월분(질유산균) + 철분 헤모케어 3포 증정</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>덴프스</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>37,050원</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000202658&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>기타/특수목적</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>[6월 올영픽/골라담기] CJ웰케어 건강루틴 가격혁명 10종 택 1</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>씨제이웰케어</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>5,900원</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000247861&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=6</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>다이어트/체중관리</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>프로뉴트리션 듀얼플랜 다이어트 유산균 14포</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>프로뉴트리션</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>33,900원</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000205496&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=7</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>다이어트/체중관리</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>솔티스 혈당/눈 프로텍션 프로S2/S3 20캡슐 (20일분)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>솔티스</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>12,900원</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000234147&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=8</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>다이어트/체중관리</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>[1등 유산균] 콜레올로지 컷 다이어트 유산균 14/20캡슐 (7/10일분)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>푸드올로지</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>18,500원</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000229934&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=9</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>멀티비타민/종합비타민</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>오쏘몰 이뮨 멀티비타민&amp;미네랄 14입 단품/기획</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>오쏘몰</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>55,900원</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000193086&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=10</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1447,32 +1790,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>전체</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>비율(%)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>카카오선물하기</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>다이소몰</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>올리브영</t>
         </is>
@@ -1485,10 +1828,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C2" t="n">
-        <v>26.7</v>
+        <v>22.5</v>
       </c>
       <c r="D2" t="n">
         <v>8</v>
@@ -1497,7 +1840,7 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -1507,10 +1850,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C3" t="n">
-        <v>6.7</v>
+        <v>7.5</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
@@ -1519,7 +1862,7 @@
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -1532,7 +1875,7 @@
         <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>3.3</v>
+        <v>2.5</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -1554,7 +1897,7 @@
         <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>3.3</v>
+        <v>2.5</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -1620,7 +1963,7 @@
         <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>3.3</v>
+        <v>2.5</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
@@ -1639,10 +1982,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C9" t="n">
-        <v>23.3</v>
+        <v>25</v>
       </c>
       <c r="D9" t="n">
         <v>6</v>
@@ -1651,7 +1994,7 @@
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -1661,10 +2004,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -1673,7 +2016,7 @@
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -1683,10 +2026,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C11" t="n">
-        <v>6.7</v>
+        <v>7.5</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
@@ -1695,7 +2038,7 @@
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -1705,10 +2048,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C12" t="n">
-        <v>26.7</v>
+        <v>27.5</v>
       </c>
       <c r="D12" t="n">
         <v>3</v>
@@ -1717,7 +2060,7 @@
         <v>5</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -1727,7 +2070,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C13" t="n">
         <v>100</v>
@@ -1739,7 +2082,7 @@
         <v>10</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>